<commit_message>
Seed ACADS weak-layer slip at base of layer (FOS 1.279 -> 1.258)
The non-circular search moves 'Horiz' points horizontally only, so the seed
elevation of the two interior points is the sliding plane and is never
optimized. The benchmark seeded them at the layer center (y=26.75), which
biased the factor of safety ~1.5% high. Placing the slip just above the base
of the weak layer (y=26.55) is standard practice for a weak interlayer and
matches the ACADS/SLOPE/W reference.

New non-circular results (ref ~1.26): Spencer 1.258 (was 1.279, now within
0.3% of SLOPE/W's 1.261), Janbu 1.278, Lowe 1.249, Corps 1.336. Updated
build_lem.py, regenerated the input xlsx and figures, refreshed the per-method
tables/tags in samples.md, verification.md, and benchmark-run-plan.md, and
added a y-sweep diagnostic (exp_weak_layer_y.py).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_acads_weak_layer.xlsx
+++ b/docs/lem/files/xslope_acads_weak_layer.xlsx
@@ -16125,7 +16125,7 @@
         <v>44</v>
       </c>
       <c r="B4" s="3">
-        <v>26.75</v>
+        <v>26.55</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -16144,7 +16144,7 @@
         <v>66</v>
       </c>
       <c r="B5" s="3">
-        <v>26.75</v>
+        <v>26.55</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>

</xml_diff>